<commit_message>
test: regenerate small fixture packages and deterministic manifest
</commit_message>
<xml_diff>
--- a/tests/fixtures/xlsx-viewer/f5-small.xlsx
+++ b/tests/fixtures/xlsx-viewer/f5-small.xlsx
@@ -55,31 +55,53 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D1">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2">
       <c r="C2">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
       <c r="B3">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D4">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
-    <row r="5" hidden="1"/>
+    <row r="5">
+      <c r="A5" t="inlineStr" s="1">
+        <is>
+          <t>head-0</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr" s="1">
+        <is>
+          <t>head-1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr" s="1">
+        <is>
+          <t>head-2</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr" s="1">
+        <is>
+          <t>head-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" hidden="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B2"/>

</xml_diff>